<commit_message>
Update samplesheet barcode77 -> barcode84
Actually barcode 84 was used instaead of barcode 77
Update sample sheet and report.
</commit_message>
<xml_diff>
--- a/data/Pilot sample summary.xlsx
+++ b/data/Pilot sample summary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11122"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unioxfordnexus-my.sharepoint.com/personal/psyc1895_ox_ac_uk/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/osama/Documents/projects/bd2_pilot/analysis/01_primary/demux_reads/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{0B8B9B76-6AA5-40EF-8C17-6564ECD6DBC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6FE0ADCE-0A83-4E23-80F1-F07AA4C01891}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15D95BAA-716A-9546-8BA4-07387F7BE8A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{D16AA900-C7CC-42F7-ACBF-B31717BAF978}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="51200" windowHeight="28800" xr2:uid="{D16AA900-C7CC-42F7-ACBF-B31717BAF978}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,9 +34,6 @@
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
-    </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
@@ -473,7 +470,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -515,13 +512,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -530,22 +523,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -570,7 +547,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -579,32 +555,32 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -943,52 +919,52 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AB55"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:AB50"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="21.54296875" style="7" customWidth="1"/>
-    <col min="3" max="3" width="23.08984375" customWidth="1"/>
-    <col min="4" max="4" width="16.26953125" customWidth="1"/>
-    <col min="5" max="5" width="20.08984375" customWidth="1"/>
+    <col min="2" max="2" width="21.5" style="7" customWidth="1"/>
+    <col min="3" max="3" width="23.1640625" customWidth="1"/>
+    <col min="4" max="4" width="16.33203125" customWidth="1"/>
+    <col min="5" max="5" width="20.1640625" customWidth="1"/>
     <col min="8" max="8" width="15" customWidth="1"/>
-    <col min="9" max="9" width="21.6328125" customWidth="1"/>
-    <col min="10" max="10" width="46.1796875" customWidth="1"/>
+    <col min="9" max="9" width="21.6640625" customWidth="1"/>
+    <col min="10" max="10" width="46.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="44" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="33" t="s">
+    <row r="1" spans="1:10" ht="49" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="25" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="25" t="s">
         <v>47</v>
       </c>
-      <c r="C1" s="34" t="s">
+      <c r="C1" s="26" t="s">
         <v>48</v>
       </c>
-      <c r="D1" s="34" t="s">
+      <c r="D1" s="26" t="s">
         <v>49</v>
       </c>
-      <c r="E1" s="34" t="s">
+      <c r="E1" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="F1" s="35" t="s">
+      <c r="F1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="G1" s="34" t="s">
+      <c r="G1" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="34" t="s">
+      <c r="H1" s="26" t="s">
         <v>56</v>
       </c>
-      <c r="I1" s="28" t="s">
+      <c r="I1" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="J1" s="37" t="s">
+      <c r="J1" s="28" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A2" s="46">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A2" s="32">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -1012,13 +988,13 @@
       <c r="H2" s="4">
         <v>13.7</v>
       </c>
-      <c r="I2" s="29" t="s">
+      <c r="I2" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="J2" s="38"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A3" s="47"/>
+      <c r="J2" s="29"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3" s="33"/>
       <c r="B3" s="6" t="s">
         <v>6</v>
       </c>
@@ -1040,13 +1016,13 @@
       <c r="H3" s="8">
         <v>12.7</v>
       </c>
-      <c r="I3" s="21" t="s">
+      <c r="I3" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="J3" s="20"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A4" s="47"/>
+      <c r="J3" s="18"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A4" s="33"/>
       <c r="B4" s="6" t="s">
         <v>7</v>
       </c>
@@ -1068,13 +1044,13 @@
       <c r="H4" s="8">
         <v>20.399999999999999</v>
       </c>
-      <c r="I4" s="21" t="s">
+      <c r="I4" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="J4" s="20"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A5" s="47"/>
+      <c r="J4" s="18"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A5" s="33"/>
       <c r="B5" s="6" t="s">
         <v>9</v>
       </c>
@@ -1096,13 +1072,13 @@
       <c r="H5" s="8">
         <v>15.3</v>
       </c>
-      <c r="I5" s="21" t="s">
+      <c r="I5" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="J5" s="20"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A6" s="47"/>
+      <c r="J5" s="18"/>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A6" s="33"/>
       <c r="B6" s="6" t="s">
         <v>11</v>
       </c>
@@ -1124,13 +1100,13 @@
       <c r="H6" s="8">
         <v>10.3</v>
       </c>
-      <c r="I6" s="21" t="s">
+      <c r="I6" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="J6" s="20"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A7" s="47"/>
+      <c r="J6" s="18"/>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A7" s="33"/>
       <c r="B7" s="6">
         <v>5298</v>
       </c>
@@ -1152,13 +1128,13 @@
       <c r="H7" s="8">
         <v>24.6</v>
       </c>
-      <c r="I7" s="21" t="s">
+      <c r="I7" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="J7" s="20"/>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A8" s="47"/>
+      <c r="J7" s="18"/>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A8" s="33"/>
       <c r="B8" s="6" t="s">
         <v>17</v>
       </c>
@@ -1180,13 +1156,13 @@
       <c r="H8" s="8">
         <v>22.2</v>
       </c>
-      <c r="I8" s="21" t="s">
+      <c r="I8" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="J8" s="20"/>
-    </row>
-    <row r="9" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="47"/>
+      <c r="J8" s="18"/>
+    </row>
+    <row r="9" spans="1:10" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="33"/>
       <c r="B9" s="11" t="s">
         <v>20</v>
       </c>
@@ -1208,13 +1184,13 @@
       <c r="H9" s="12">
         <v>23.8</v>
       </c>
-      <c r="I9" s="30" t="s">
+      <c r="I9" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="J9" s="39"/>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A10" s="46">
+      <c r="J9" s="30"/>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A10" s="32">
         <v>2</v>
       </c>
       <c r="B10" s="3" t="s">
@@ -1238,13 +1214,13 @@
       <c r="H10" s="4">
         <v>60.2</v>
       </c>
-      <c r="I10" s="31" t="s">
+      <c r="I10" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="J10" s="20"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A11" s="47"/>
+      <c r="J10" s="18"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A11" s="33"/>
       <c r="B11" s="6" t="s">
         <v>42</v>
       </c>
@@ -1266,155 +1242,155 @@
       <c r="H11" s="8">
         <v>9.66</v>
       </c>
-      <c r="I11" s="21" t="s">
+      <c r="I11" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="J11" s="20" t="s">
+      <c r="J11" s="18" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A12" s="47"/>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A12" s="33"/>
       <c r="B12" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="C12" s="15" t="s">
+      <c r="C12" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D12" s="15" t="s">
+      <c r="D12" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="E12" s="15" t="s">
+      <c r="E12" s="8" t="s">
         <v>5</v>
       </c>
       <c r="F12" s="9">
         <v>8.6999999999999993</v>
       </c>
-      <c r="G12" s="15">
+      <c r="G12" s="8">
         <v>52</v>
       </c>
-      <c r="H12" s="15">
+      <c r="H12" s="8">
         <v>72</v>
       </c>
-      <c r="I12" s="31" t="s">
+      <c r="I12" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="J12" s="20"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A13" s="47"/>
+      <c r="J12" s="18"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A13" s="33"/>
       <c r="B13" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="C13" s="15" t="s">
+      <c r="C13" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D13" s="15" t="s">
+      <c r="D13" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E13" s="15" t="s">
+      <c r="E13" s="8" t="s">
         <v>5</v>
       </c>
       <c r="F13" s="9">
         <v>8.1999999999999993</v>
       </c>
-      <c r="G13" s="22">
+      <c r="G13" s="15">
         <v>70</v>
       </c>
       <c r="H13" s="8">
         <v>61</v>
       </c>
-      <c r="I13" s="31" t="s">
+      <c r="I13" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="J13" s="20"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A14" s="47"/>
+      <c r="J13" s="18"/>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A14" s="33"/>
       <c r="B14" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C14" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D14" s="15" t="s">
+      <c r="D14" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E14" s="15" t="s">
+      <c r="E14" s="8" t="s">
         <v>14</v>
       </c>
       <c r="F14" s="9">
         <v>5.7</v>
       </c>
-      <c r="G14" s="15">
+      <c r="G14" s="8">
         <v>63</v>
       </c>
-      <c r="H14" s="15">
+      <c r="H14" s="8">
         <v>56.8</v>
       </c>
-      <c r="I14" s="31" t="s">
+      <c r="I14" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="J14" s="20"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A15" s="47"/>
+      <c r="J14" s="18"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A15" s="33"/>
       <c r="B15" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C15" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D15" s="15" t="s">
+      <c r="D15" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E15" s="15" t="s">
+      <c r="E15" s="8" t="s">
         <v>14</v>
       </c>
       <c r="F15" s="9">
         <v>6.6</v>
       </c>
-      <c r="G15" s="15">
+      <c r="G15" s="8">
         <v>66</v>
       </c>
-      <c r="H15" s="15">
+      <c r="H15" s="8">
         <v>53.8</v>
       </c>
-      <c r="I15" s="31" t="s">
+      <c r="I15" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="J15" s="20"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
-      <c r="A16" s="47"/>
+      <c r="J15" s="18"/>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A16" s="33"/>
       <c r="B16" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="15" t="s">
+      <c r="C16" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="D16" s="15" t="s">
+      <c r="D16" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E16" s="15" t="s">
+      <c r="E16" s="8" t="s">
         <v>14</v>
       </c>
       <c r="F16" s="9">
         <v>5.5</v>
       </c>
-      <c r="G16" s="15">
+      <c r="G16" s="8">
         <v>61</v>
       </c>
-      <c r="H16" s="15">
+      <c r="H16" s="8">
         <v>61</v>
       </c>
-      <c r="I16" s="31" t="s">
+      <c r="I16" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="J16" s="20"/>
-    </row>
-    <row r="17" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="48"/>
+      <c r="J16" s="18"/>
+    </row>
+    <row r="17" spans="1:28" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="34"/>
       <c r="B17" s="11" t="s">
         <v>19</v>
       </c>
@@ -1436,13 +1412,13 @@
       <c r="H17" s="12">
         <v>54.8</v>
       </c>
-      <c r="I17" s="32" t="s">
+      <c r="I17" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="J17" s="39"/>
-    </row>
-    <row r="18" spans="1:28" x14ac:dyDescent="0.35">
-      <c r="A18" s="46">
+      <c r="J17" s="30"/>
+    </row>
+    <row r="18" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A18" s="32">
         <v>3</v>
       </c>
       <c r="B18" s="3" t="s">
@@ -1466,109 +1442,109 @@
       <c r="H18" s="4">
         <v>97.2</v>
       </c>
-      <c r="I18" s="31" t="s">
+      <c r="I18" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="J18" s="20"/>
+      <c r="J18" s="18"/>
       <c r="AB18" s="1"/>
     </row>
-    <row r="19" spans="1:28" x14ac:dyDescent="0.35">
-      <c r="A19" s="47"/>
+    <row r="19" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A19" s="33"/>
       <c r="B19" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="C19" s="15" t="s">
+      <c r="C19" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D19" s="15" t="s">
+      <c r="D19" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="E19" s="15" t="s">
+      <c r="E19" s="8" t="s">
         <v>5</v>
       </c>
       <c r="F19" s="9">
         <v>8.5</v>
       </c>
-      <c r="G19" s="15">
+      <c r="G19" s="8">
         <v>67</v>
       </c>
-      <c r="H19" s="15">
+      <c r="H19" s="8">
         <v>48.5</v>
       </c>
-      <c r="I19" s="31" t="s">
+      <c r="I19" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="J19" s="20"/>
+      <c r="J19" s="18"/>
       <c r="AB19" s="1"/>
     </row>
-    <row r="20" spans="1:28" x14ac:dyDescent="0.35">
-      <c r="A20" s="47"/>
+    <row r="20" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A20" s="33"/>
       <c r="B20" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="C20" s="15" t="s">
+      <c r="C20" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D20" s="15" t="s">
+      <c r="D20" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E20" s="15" t="s">
+      <c r="E20" s="8" t="s">
         <v>5</v>
       </c>
       <c r="F20" s="9">
         <v>8.1999999999999993</v>
       </c>
-      <c r="G20" s="15">
+      <c r="G20" s="8">
         <v>76</v>
       </c>
-      <c r="H20" s="15">
+      <c r="H20" s="8">
         <v>21.6</v>
       </c>
-      <c r="I20" s="31" t="s">
+      <c r="I20" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="J20" s="20"/>
-    </row>
-    <row r="21" spans="1:28" x14ac:dyDescent="0.35">
-      <c r="A21" s="47"/>
+      <c r="J20" s="18"/>
+    </row>
+    <row r="21" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A21" s="33"/>
       <c r="B21" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="C21" s="15" t="s">
+      <c r="C21" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D21" s="15" t="s">
+      <c r="D21" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="E21" s="15" t="s">
+      <c r="E21" s="8" t="s">
         <v>5</v>
       </c>
       <c r="F21" s="9">
         <v>8.3000000000000007</v>
       </c>
-      <c r="G21" s="15">
+      <c r="G21" s="8">
         <v>68</v>
       </c>
-      <c r="H21" s="15">
+      <c r="H21" s="8">
         <v>39.1</v>
       </c>
-      <c r="I21" s="31" t="s">
+      <c r="I21" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="J21" s="20"/>
-    </row>
-    <row r="22" spans="1:28" x14ac:dyDescent="0.35">
-      <c r="A22" s="47"/>
+      <c r="J21" s="18"/>
+    </row>
+    <row r="22" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A22" s="33"/>
       <c r="B22" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C22" s="15" t="s">
+      <c r="C22" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="D22" s="15" t="s">
+      <c r="D22" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E22" s="15" t="s">
+      <c r="E22" s="8" t="s">
         <v>14</v>
       </c>
       <c r="F22" s="9">
@@ -1580,23 +1556,23 @@
       <c r="H22" s="8">
         <v>25.2</v>
       </c>
-      <c r="I22" s="31" t="s">
+      <c r="I22" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="J22" s="20"/>
-    </row>
-    <row r="23" spans="1:28" x14ac:dyDescent="0.35">
-      <c r="A23" s="47"/>
+      <c r="J22" s="18"/>
+    </row>
+    <row r="23" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A23" s="33"/>
       <c r="B23" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C23" s="15" t="s">
+      <c r="C23" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="D23" s="15" t="s">
+      <c r="D23" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E23" s="15" t="s">
+      <c r="E23" s="8" t="s">
         <v>14</v>
       </c>
       <c r="F23" s="9">
@@ -1608,23 +1584,23 @@
       <c r="H23" s="8">
         <v>36.4</v>
       </c>
-      <c r="I23" s="31" t="s">
+      <c r="I23" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="J23" s="20"/>
-    </row>
-    <row r="24" spans="1:28" x14ac:dyDescent="0.35">
-      <c r="A24" s="47"/>
+      <c r="J23" s="18"/>
+    </row>
+    <row r="24" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A24" s="33"/>
       <c r="B24" s="6" t="s">
         <v>36</v>
       </c>
       <c r="C24" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D24" s="15" t="s">
+      <c r="D24" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E24" s="15" t="s">
+      <c r="E24" s="8" t="s">
         <v>14</v>
       </c>
       <c r="F24" s="9">
@@ -1636,13 +1612,13 @@
       <c r="H24" s="8">
         <v>54.4</v>
       </c>
-      <c r="I24" s="31" t="s">
+      <c r="I24" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="J24" s="20"/>
-    </row>
-    <row r="25" spans="1:28" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A25" s="48"/>
+      <c r="J24" s="18"/>
+    </row>
+    <row r="25" spans="1:28" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="34"/>
       <c r="B25" s="11" t="s">
         <v>21</v>
       </c>
@@ -1664,15 +1640,15 @@
       <c r="H25" s="12">
         <v>47.6</v>
       </c>
-      <c r="I25" s="32" t="s">
+      <c r="I25" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="J25" s="39" t="s">
+      <c r="J25" s="30" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="26" spans="1:28" x14ac:dyDescent="0.35">
-      <c r="A26" s="46">
+    <row r="26" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A26" s="32">
         <v>4</v>
       </c>
       <c r="B26" s="6" t="s">
@@ -1696,15 +1672,15 @@
       <c r="H26" s="8">
         <v>13.5</v>
       </c>
-      <c r="I26" s="21" t="s">
+      <c r="I26" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="J26" s="20" t="s">
+      <c r="J26" s="18" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="27" spans="1:28" x14ac:dyDescent="0.35">
-      <c r="A27" s="47"/>
+    <row r="27" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A27" s="33"/>
       <c r="B27" s="6" t="s">
         <v>44</v>
       </c>
@@ -1726,83 +1702,83 @@
       <c r="H27" s="8">
         <v>21</v>
       </c>
-      <c r="I27" s="21" t="s">
+      <c r="I27" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="J27" s="20" t="s">
+      <c r="J27" s="18" t="s">
         <v>62</v>
       </c>
       <c r="K27" s="8"/>
       <c r="L27" s="8"/>
     </row>
-    <row r="28" spans="1:28" x14ac:dyDescent="0.35">
-      <c r="A28" s="47"/>
+    <row r="28" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A28" s="33"/>
       <c r="B28" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="C28" s="15" t="s">
+      <c r="C28" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D28" s="15" t="s">
+      <c r="D28" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="E28" s="15" t="s">
+      <c r="E28" s="8" t="s">
         <v>5</v>
       </c>
       <c r="F28" s="9">
         <v>8.9</v>
       </c>
-      <c r="G28" s="15">
+      <c r="G28" s="8">
         <v>53</v>
       </c>
-      <c r="H28" s="15">
+      <c r="H28" s="8">
         <v>73.400000000000006</v>
       </c>
-      <c r="I28" s="31" t="s">
+      <c r="I28" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="J28" s="20"/>
-    </row>
-    <row r="29" spans="1:28" x14ac:dyDescent="0.35">
-      <c r="A29" s="47"/>
+      <c r="J28" s="18"/>
+    </row>
+    <row r="29" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A29" s="33"/>
       <c r="B29" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="C29" s="15" t="s">
+      <c r="C29" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D29" s="15" t="s">
+      <c r="D29" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E29" s="15" t="s">
+      <c r="E29" s="8" t="s">
         <v>5</v>
       </c>
       <c r="F29" s="9">
         <v>8.1</v>
       </c>
-      <c r="G29" s="16">
+      <c r="G29" s="15">
         <v>74</v>
       </c>
-      <c r="H29" s="15">
+      <c r="H29" s="8">
         <v>26.5</v>
       </c>
-      <c r="I29" s="31" t="s">
+      <c r="I29" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="J29" s="20"/>
-    </row>
-    <row r="30" spans="1:28" x14ac:dyDescent="0.35">
-      <c r="A30" s="47"/>
+      <c r="J29" s="18"/>
+    </row>
+    <row r="30" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A30" s="33"/>
       <c r="B30" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="C30" s="15" t="s">
+      <c r="C30" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D30" s="15" t="s">
+      <c r="D30" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E30" s="15" t="s">
+      <c r="E30" s="8" t="s">
         <v>5</v>
       </c>
       <c r="F30" s="9">
@@ -1814,23 +1790,23 @@
       <c r="H30" s="8">
         <v>46.8</v>
       </c>
-      <c r="I30" s="31" t="s">
+      <c r="I30" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="J30" s="20"/>
-    </row>
-    <row r="31" spans="1:28" x14ac:dyDescent="0.35">
-      <c r="A31" s="47"/>
+      <c r="J30" s="18"/>
+    </row>
+    <row r="31" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A31" s="33"/>
       <c r="B31" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C31" s="15" t="s">
+      <c r="C31" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D31" s="15" t="s">
+      <c r="D31" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E31" s="15" t="s">
+      <c r="E31" s="8" t="s">
         <v>14</v>
       </c>
       <c r="F31" s="9">
@@ -1842,41 +1818,41 @@
       <c r="H31" s="8">
         <v>32.6</v>
       </c>
-      <c r="I31" s="31" t="s">
+      <c r="I31" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="J31" s="20"/>
-    </row>
-    <row r="32" spans="1:28" x14ac:dyDescent="0.35">
-      <c r="A32" s="47"/>
+      <c r="J31" s="18"/>
+    </row>
+    <row r="32" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A32" s="33"/>
       <c r="B32" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C32" s="15" t="s">
+      <c r="C32" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="D32" s="15" t="s">
+      <c r="D32" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E32" s="15" t="s">
+      <c r="E32" s="8" t="s">
         <v>14</v>
       </c>
       <c r="F32" s="9">
         <v>4.8</v>
       </c>
-      <c r="G32" s="15">
+      <c r="G32" s="8">
         <v>64</v>
       </c>
-      <c r="H32" s="15">
+      <c r="H32" s="8">
         <v>90.6</v>
       </c>
-      <c r="I32" s="31" t="s">
+      <c r="I32" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="J32" s="20"/>
-    </row>
-    <row r="33" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A33" s="48"/>
+      <c r="J32" s="18"/>
+    </row>
+    <row r="33" spans="1:12" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="34"/>
       <c r="B33" s="11" t="s">
         <v>21</v>
       </c>
@@ -1898,13 +1874,13 @@
       <c r="H33" s="12">
         <v>40.799999999999997</v>
       </c>
-      <c r="I33" s="32" t="s">
+      <c r="I33" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="J33" s="39"/>
-    </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A34" s="46">
+      <c r="J33" s="30"/>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A34" s="32">
         <v>5</v>
       </c>
       <c r="B34" s="2" t="s">
@@ -1923,90 +1899,87 @@
         <v>8.4</v>
       </c>
       <c r="G34" s="4">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="H34" s="4">
         <v>54.4</v>
       </c>
-      <c r="I34" s="31" t="s">
+      <c r="I34" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="J34" s="20"/>
-    </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A35" s="47"/>
+      <c r="J34" s="18"/>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A35" s="33"/>
       <c r="B35" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="C35" s="15" t="s">
+      <c r="C35" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D35" s="15" t="s">
+      <c r="D35" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="E35" s="15" t="s">
+      <c r="E35" s="8" t="s">
         <v>5</v>
       </c>
       <c r="F35" s="9">
         <v>8.6</v>
       </c>
-      <c r="G35" s="15">
+      <c r="G35" s="8">
         <v>73</v>
       </c>
-      <c r="H35" s="15">
+      <c r="H35" s="8">
         <v>70.5</v>
       </c>
-      <c r="I35" s="31" t="s">
+      <c r="I35" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="J35" s="20"/>
-    </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A36" s="47"/>
+      <c r="J35" s="18"/>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A36" s="33"/>
       <c r="B36" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="C36" s="15" t="s">
+      <c r="C36" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D36" s="15" t="s">
+      <c r="D36" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="E36" s="15" t="s">
+      <c r="E36" s="8" t="s">
         <v>5</v>
       </c>
       <c r="F36" s="9">
         <v>9.1</v>
       </c>
-      <c r="G36" s="15">
+      <c r="G36" s="8">
         <v>75</v>
       </c>
-      <c r="H36" s="15">
+      <c r="H36" s="8">
         <v>82.9</v>
       </c>
-      <c r="I36" s="31" t="s">
+      <c r="I36" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="J36" s="20"/>
-      <c r="K36" s="17"/>
-      <c r="L36" s="17"/>
-      <c r="M36" s="17"/>
-    </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A37" s="47"/>
+      <c r="J36" s="18"/>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A37" s="33"/>
       <c r="B37" s="6" t="s">
         <v>45</v>
       </c>
       <c r="C37" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D37" s="23" t="s">
+      <c r="D37" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E37" s="23" t="s">
+      <c r="E37" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F37" s="24">
+      <c r="F37" s="9">
         <v>6.5</v>
       </c>
       <c r="G37" s="8">
@@ -2018,89 +1991,85 @@
       <c r="I37" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="J37" s="20" t="s">
+      <c r="J37" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="K37" s="15"/>
-      <c r="L37" s="15"/>
-      <c r="M37" s="17"/>
-    </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A38" s="49"/>
+      <c r="K37" s="8"/>
+      <c r="L37" s="8"/>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A38" s="37"/>
       <c r="B38" s="6" t="s">
         <v>46</v>
       </c>
       <c r="C38" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D38" s="25" t="s">
+      <c r="D38" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E38" s="25" t="s">
+      <c r="E38" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="F38" s="24">
+      <c r="F38" s="9">
         <v>6.5</v>
       </c>
-      <c r="G38" s="15">
+      <c r="G38" s="8">
         <v>57</v>
       </c>
-      <c r="H38" s="15">
+      <c r="H38" s="8">
         <v>36</v>
       </c>
-      <c r="I38" s="21" t="s">
+      <c r="I38" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="J38" s="20" t="s">
+      <c r="J38" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="K38" s="17"/>
-      <c r="L38" s="17"/>
-      <c r="M38" s="17"/>
-    </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A39" s="49"/>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A39" s="37"/>
       <c r="B39" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="C39" s="25" t="s">
+      <c r="C39" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="D39" s="25" t="s">
+      <c r="D39" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="E39" s="25" t="s">
+      <c r="E39" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="F39" s="24">
+      <c r="F39" s="9">
         <v>8.5</v>
       </c>
-      <c r="G39" s="15">
+      <c r="G39" s="8">
         <v>71</v>
       </c>
-      <c r="H39" s="15">
+      <c r="H39" s="8">
         <v>44</v>
       </c>
-      <c r="I39" s="31" t="s">
+      <c r="I39" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="J39" s="20"/>
-    </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A40" s="47"/>
+      <c r="J39" s="18"/>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A40" s="33"/>
       <c r="B40" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="C40" s="25" t="s">
+      <c r="C40" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="D40" s="25" t="s">
+      <c r="D40" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="E40" s="25" t="s">
+      <c r="E40" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="F40" s="24">
+      <c r="F40" s="9">
         <v>8.1999999999999993</v>
       </c>
       <c r="G40" s="8">
@@ -2109,14 +2078,14 @@
       <c r="H40" s="8">
         <v>80.8</v>
       </c>
-      <c r="I40" s="31" t="s">
+      <c r="I40" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="J40" s="20"/>
-    </row>
-    <row r="41" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A41" s="48"/>
-      <c r="B41" s="18" t="s">
+      <c r="J40" s="18"/>
+    </row>
+    <row r="41" spans="1:12" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="34"/>
+      <c r="B41" s="16" t="s">
         <v>29</v>
       </c>
       <c r="C41" s="12" t="s">
@@ -2137,162 +2106,97 @@
       <c r="H41" s="12">
         <v>20</v>
       </c>
-      <c r="I41" s="32" t="s">
+      <c r="I41" s="24" t="s">
         <v>53</v>
       </c>
-      <c r="J41" s="39"/>
-    </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A43" s="26"/>
-      <c r="B43" s="45" t="s">
+      <c r="J41" s="30"/>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="B43" s="35" t="s">
         <v>57</v>
       </c>
-      <c r="C43" s="45"/>
-      <c r="D43" s="45"/>
-      <c r="E43" s="45"/>
-      <c r="F43" s="45"/>
-      <c r="G43" s="45"/>
-      <c r="H43" s="45"/>
-      <c r="I43" s="45"/>
-    </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A44" s="26"/>
-      <c r="B44" s="43" t="s">
+      <c r="C43" s="35"/>
+      <c r="D43" s="35"/>
+      <c r="E43" s="35"/>
+      <c r="F43" s="35"/>
+      <c r="G43" s="35"/>
+      <c r="H43" s="35"/>
+      <c r="I43" s="35"/>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="B44" s="36" t="s">
         <v>53</v>
       </c>
-      <c r="C44" s="43"/>
-      <c r="D44" s="43" t="s">
+      <c r="C44" s="36"/>
+      <c r="D44" s="36" t="s">
         <v>58</v>
       </c>
-      <c r="E44" s="43"/>
-      <c r="F44" s="43"/>
-      <c r="G44" s="43"/>
-      <c r="H44" s="43"/>
-      <c r="I44" s="43"/>
-    </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A45" s="26"/>
-      <c r="B45" s="43" t="s">
+      <c r="E44" s="36"/>
+      <c r="F44" s="36"/>
+      <c r="G44" s="36"/>
+      <c r="H44" s="36"/>
+      <c r="I44" s="36"/>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="B45" s="36" t="s">
         <v>51</v>
       </c>
-      <c r="C45" s="43"/>
-      <c r="D45" s="43" t="s">
+      <c r="C45" s="36"/>
+      <c r="D45" s="36" t="s">
         <v>60</v>
       </c>
-      <c r="E45" s="43"/>
-      <c r="F45" s="43"/>
-      <c r="G45" s="43"/>
-      <c r="H45" s="43"/>
-      <c r="I45" s="43"/>
-    </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A46" s="26"/>
-      <c r="B46" s="44" t="s">
+      <c r="E45" s="36"/>
+      <c r="F45" s="36"/>
+      <c r="G45" s="36"/>
+      <c r="H45" s="36"/>
+      <c r="I45" s="36"/>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="B46" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="C46" s="44"/>
-      <c r="D46" s="43" t="s">
+      <c r="C46" s="40"/>
+      <c r="D46" s="36" t="s">
         <v>59</v>
       </c>
-      <c r="E46" s="43"/>
-      <c r="F46" s="43"/>
-      <c r="G46" s="43"/>
-      <c r="H46" s="43"/>
-      <c r="I46" s="43"/>
-    </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A47" s="26"/>
-      <c r="B47" s="25"/>
-      <c r="C47" s="26"/>
-      <c r="D47" s="26"/>
-      <c r="E47" s="26"/>
-      <c r="F47" s="26"/>
-    </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.35">
-      <c r="A48" s="26"/>
-      <c r="C48" s="42" t="s">
+      <c r="E46" s="36"/>
+      <c r="F46" s="36"/>
+      <c r="G46" s="36"/>
+      <c r="H46" s="36"/>
+      <c r="I46" s="36"/>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="B47" s="8"/>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="C48" s="39" t="s">
         <v>64</v>
       </c>
-      <c r="D48" s="42"/>
-      <c r="E48" s="42"/>
-      <c r="F48" s="42"/>
-      <c r="G48" s="42"/>
-      <c r="H48" s="42"/>
-      <c r="I48" s="42"/>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A49" s="26"/>
-      <c r="C49" s="40" t="s">
+      <c r="D48" s="39"/>
+      <c r="E48" s="39"/>
+      <c r="F48" s="39"/>
+      <c r="G48" s="39"/>
+      <c r="H48" s="39"/>
+      <c r="I48" s="39"/>
+    </row>
+    <row r="49" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="C49" s="31" t="s">
         <v>66</v>
       </c>
-      <c r="D49" s="41" t="s">
+      <c r="D49" s="38" t="s">
         <v>65</v>
       </c>
-      <c r="E49" s="41"/>
-      <c r="F49" s="41"/>
-      <c r="G49" s="41"/>
-      <c r="H49" s="41"/>
-      <c r="I49" s="41"/>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A50" s="26"/>
-      <c r="B50" s="36"/>
-      <c r="C50" s="36"/>
-      <c r="D50" s="36"/>
-      <c r="E50" s="36"/>
-      <c r="F50" s="36"/>
-      <c r="G50" s="36"/>
-      <c r="H50" s="36"/>
-      <c r="I50" s="36"/>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A51" s="26"/>
-      <c r="B51" s="27"/>
-      <c r="C51" s="26"/>
-      <c r="D51" s="26"/>
-      <c r="E51" s="26"/>
-      <c r="F51" s="26"/>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A52" s="26"/>
-      <c r="B52" s="27"/>
-      <c r="C52" s="26"/>
-      <c r="D52" s="26"/>
-      <c r="E52" s="26"/>
-      <c r="F52" s="26"/>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A53" s="26"/>
-      <c r="B53" s="27"/>
-      <c r="C53" s="26"/>
-      <c r="D53" s="26"/>
-      <c r="E53" s="26"/>
-      <c r="F53" s="26"/>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A54" s="26"/>
-      <c r="B54" s="27"/>
-      <c r="C54" s="26"/>
-      <c r="D54" s="26"/>
-      <c r="E54" s="26"/>
-      <c r="F54" s="26"/>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A55" s="26"/>
-      <c r="B55" s="27"/>
-      <c r="C55" s="26"/>
-      <c r="D55" s="26"/>
-      <c r="E55" s="26"/>
-      <c r="F55" s="26"/>
+      <c r="E49" s="38"/>
+      <c r="F49" s="38"/>
+      <c r="G49" s="38"/>
+      <c r="H49" s="38"/>
+      <c r="I49" s="38"/>
+    </row>
+    <row r="50" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="B50"/>
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="A2:A9"/>
-    <mergeCell ref="A10:A17"/>
-    <mergeCell ref="A18:A25"/>
-    <mergeCell ref="B43:I43"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="D44:I44"/>
     <mergeCell ref="D45:I45"/>
     <mergeCell ref="A26:A33"/>
     <mergeCell ref="A34:A41"/>
@@ -2301,6 +2205,12 @@
     <mergeCell ref="D46:I46"/>
     <mergeCell ref="B45:C45"/>
     <mergeCell ref="B46:C46"/>
+    <mergeCell ref="A2:A9"/>
+    <mergeCell ref="A10:A17"/>
+    <mergeCell ref="A18:A25"/>
+    <mergeCell ref="B43:I43"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="D44:I44"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2311,148 +2221,148 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFEC1EB3-E65C-4CBE-BA16-FC94EC7649B1}">
   <dimension ref="B3:C18"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B3">
         <v>97.2</v>
       </c>
-      <c r="C3" s="19">
+      <c r="C3" s="17">
         <f>150/B3</f>
         <v>1.5432098765432098</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B4">
         <v>48.5</v>
       </c>
-      <c r="C4" s="19">
+      <c r="C4" s="17">
         <f t="shared" ref="C4:C18" si="0">150/B4</f>
         <v>3.0927835051546393</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B5">
         <v>21.6</v>
       </c>
-      <c r="C5" s="19">
+      <c r="C5" s="17">
         <f t="shared" si="0"/>
         <v>6.9444444444444438</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B6">
         <v>39.1</v>
       </c>
-      <c r="C6" s="19">
+      <c r="C6" s="17">
         <f t="shared" si="0"/>
         <v>3.836317135549872</v>
       </c>
     </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B7">
         <v>25.2</v>
       </c>
-      <c r="C7" s="19">
+      <c r="C7" s="17">
         <f t="shared" si="0"/>
         <v>5.9523809523809526</v>
       </c>
     </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B8">
         <v>36.4</v>
       </c>
-      <c r="C8" s="19">
+      <c r="C8" s="17">
         <f t="shared" si="0"/>
         <v>4.1208791208791213</v>
       </c>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B9">
         <v>54.4</v>
       </c>
-      <c r="C9" s="19">
+      <c r="C9" s="17">
         <f t="shared" si="0"/>
         <v>2.7573529411764706</v>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B10">
         <v>47.6</v>
       </c>
-      <c r="C10" s="19">
+      <c r="C10" s="17">
         <f t="shared" si="0"/>
         <v>3.1512605042016806</v>
       </c>
     </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B11">
         <v>54.4</v>
       </c>
-      <c r="C11" s="19">
+      <c r="C11" s="17">
         <f t="shared" si="0"/>
         <v>2.7573529411764706</v>
       </c>
     </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B12">
         <v>70.5</v>
       </c>
-      <c r="C12" s="19">
+      <c r="C12" s="17">
         <f t="shared" si="0"/>
         <v>2.1276595744680851</v>
       </c>
     </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B13">
         <v>82.9</v>
       </c>
-      <c r="C13" s="19">
+      <c r="C13" s="17">
         <f t="shared" si="0"/>
         <v>1.8094089264173703</v>
       </c>
     </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B14">
         <v>89.2</v>
       </c>
-      <c r="C14" s="19">
+      <c r="C14" s="17">
         <f t="shared" si="0"/>
         <v>1.6816143497757847</v>
       </c>
     </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B15">
         <v>67</v>
       </c>
-      <c r="C15" s="19">
+      <c r="C15" s="17">
         <f t="shared" si="0"/>
         <v>2.2388059701492535</v>
       </c>
     </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B16">
         <v>44</v>
       </c>
-      <c r="C16" s="19">
+      <c r="C16" s="17">
         <f t="shared" si="0"/>
         <v>3.4090909090909092</v>
       </c>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B17">
         <v>80</v>
       </c>
-      <c r="C17" s="19">
+      <c r="C17" s="17">
         <f t="shared" si="0"/>
         <v>1.875</v>
       </c>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B18">
         <v>20</v>
       </c>
-      <c r="C18" s="19">
+      <c r="C18" s="17">
         <f t="shared" si="0"/>
         <v>7.5</v>
       </c>

</xml_diff>